<commit_message>
Update berita 2026-08-05 03:48 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-04.xlsx
+++ b/data/berita_antara_2026-08-04.xlsx
@@ -25411,33 +25411,33 @@
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>Klasemen Grup A Piala AFF 2026: Indonesia tempati posisi ketiga</t>
+          <t>Rupiah Selasa melemah dipicu kenaikan harga minyak global</t>
         </is>
       </c>
       <c r="C766" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 23:48:18 +0700</t>
+          <t>Tue, 04 Aug 2026 11:15:57 +0700</t>
         </is>
       </c>
       <c r="D766" t="inlineStr"/>
       <c r="E766" t="inlineStr">
         <is>
-          <t>Timnas Indonesia menempati posisi ketiga klasemen sementara Grup A Piala AFF 2026 setelah memainkan total tiga ...</t>
+          <t>Nilai tukar rupiah pada Selasa pagi bergerak melemah 32 poin atau 0,18 persen menjadi Rp18.029 per dolar AS ...</t>
         </is>
       </c>
       <c r="F766" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680113/klasemen-grup-a-piala-aff-2026-indonesia-tempati-posisi-ketiga</t>
+          <t>https://www.antaranews.com/berita/5678808/rupiah-selasa-melemah-dipicu-kenaikan-harga-minyak-global</t>
         </is>
       </c>
       <c r="G766" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/timnas-indonesia-dikalahkan-vietnam-di-piala-aff-2833635.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/nilai-tukar-rupiah-melemah-44-poin-2821215.jpg</t>
         </is>
       </c>
       <c r="H766" t="inlineStr">
@@ -25454,28 +25454,28 @@
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>Menhub tegaskan insiden KMP Mutiara Sentosa jadi evaluasi total</t>
+          <t>Klasemen Grup A Piala AFF 2026: Indonesia tempati posisi ketiga</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 23:48:02 +0700</t>
+          <t>Tue, 04 Aug 2026 23:48:18 +0700</t>
         </is>
       </c>
       <c r="D767" t="inlineStr"/>
       <c r="E767" t="inlineStr">
         <is>
-          <t>Menteri Perhubungan (Menhub) Dudy Purwagandhi menegaskan insiden kebakaran KMP Mutiara Sentosa II di perairan utara ...</t>
+          <t>Timnas Indonesia menempati posisi ketiga klasemen sementara Grup A Piala AFF 2026 setelah memainkan total tiga ...</t>
         </is>
       </c>
       <c r="F767" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680109/menhub-tegaskan-insiden-kmp-mutiara-sentosa-jadi-evaluasi-total</t>
+          <t>https://www.antaranews.com/berita/5680113/klasemen-grup-a-piala-aff-2026-indonesia-tempati-posisi-ketiga</t>
         </is>
       </c>
       <c r="G767" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/07DA5D4C-ACC9-4FDA-A3C3-B8FAE116FE12.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/timnas-indonesia-dikalahkan-vietnam-di-piala-aff-2833635.jpg</t>
         </is>
       </c>
       <c r="H767" t="inlineStr">
@@ -25492,28 +25492,28 @@
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>Mendikdasmen: Pembatasan gawai ciptakan lingkungan sekolah yang aman</t>
+          <t>Menhub tegaskan insiden KMP Mutiara Sentosa jadi evaluasi total</t>
         </is>
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 22:05:12 +0700</t>
+          <t>Tue, 04 Aug 2026 23:48:02 +0700</t>
         </is>
       </c>
       <c r="D768" t="inlineStr"/>
       <c r="E768" t="inlineStr">
         <is>
-          <t>Menteri Pendidikan Dasar dan Menengah (Mendikdasmen) Abdul Mu'ti mengatakan Surat Edaran (SE) Nomor 18 Tahun 2026 ...</t>
+          <t>Menteri Perhubungan (Menhub) Dudy Purwagandhi menegaskan insiden kebakaran KMP Mutiara Sentosa II di perairan utara ...</t>
         </is>
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680024/mendikdasmen-pembatasan-gawai-ciptakan-lingkungan-sekolah-yang-aman</t>
+          <t>https://www.antaranews.com/berita/5680109/menhub-tegaskan-insiden-kmp-mutiara-sentosa-jadi-evaluasi-total</t>
         </is>
       </c>
       <c r="G768" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Gernas-Rana-diperkuat-untuk-perlindungan-anak-040826-MRH-7_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/07DA5D4C-ACC9-4FDA-A3C3-B8FAE116FE12.jpeg</t>
         </is>
       </c>
       <c r="H768" t="inlineStr">
@@ -25530,28 +25530,28 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>Kebakaran hutan lindung Gunung Soputan meluas capai 300 hektare</t>
+          <t>Mendikdasmen: Pembatasan gawai ciptakan lingkungan sekolah yang aman</t>
         </is>
       </c>
       <c r="C769" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 21:44:20 +0700</t>
+          <t>Tue, 04 Aug 2026 22:05:12 +0700</t>
         </is>
       </c>
       <c r="D769" t="inlineStr"/>
       <c r="E769" t="inlineStr">
         <is>
-          <t>Kepala Bidang Kedaruratan dan Logistik Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Minahasa Tenggara, Sulawesi ...</t>
+          <t>Menteri Pendidikan Dasar dan Menengah (Mendikdasmen) Abdul Mu'ti mengatakan Surat Edaran (SE) Nomor 18 Tahun 2026 ...</t>
         </is>
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679992/kebakaran-hutan-lindung-gunung-soputan-meluas-capai-300-hektare</t>
+          <t>https://www.antaranews.com/berita/5680024/mendikdasmen-pembatasan-gawai-ciptakan-lingkungan-sekolah-yang-aman</t>
         </is>
       </c>
       <c r="G769" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001982099_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Gernas-Rana-diperkuat-untuk-perlindungan-anak-040826-MRH-7_1.jpg</t>
         </is>
       </c>
       <c r="H769" t="inlineStr">
@@ -25568,28 +25568,28 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>Indonesia tambah tiga medali pada hari keempat Indonesia Open</t>
+          <t>Kebakaran hutan lindung Gunung Soputan meluas capai 300 hektare</t>
         </is>
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 21:43:26 +0700</t>
+          <t>Tue, 04 Aug 2026 21:44:20 +0700</t>
         </is>
       </c>
       <c r="D770" t="inlineStr"/>
       <c r="E770" t="inlineStr">
         <is>
-          <t>Indonesia menambah tiga medali yang terdiri dari satu perak dan dua perunggu pada hari keempat 8th Asian Taekwondo ...</t>
+          <t>Kepala Bidang Kedaruratan dan Logistik Badan Penanggulangan Bencana Daerah (BPBD) Kabupaten Minahasa Tenggara, Sulawesi ...</t>
         </is>
       </c>
       <c r="F770" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679989/indonesia-tambah-tiga-medali-pada-hari-keempat-indonesia-open</t>
+          <t>https://www.antaranews.com/berita/5679992/kebakaran-hutan-lindung-gunung-soputan-meluas-capai-300-hektare</t>
         </is>
       </c>
       <c r="G770" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/adrian-kaiser-raih-perak-asian-taekwondo-indonesia-open-championships-2834348.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1001982099_1.jpg</t>
         </is>
       </c>
       <c r="H770" t="inlineStr">
@@ -25606,28 +25606,28 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>KPK tahan tiga tersangka kasus dugaan korupsi dalam digitalisasi SPBU</t>
+          <t>Indonesia tambah tiga medali pada hari keempat Indonesia Open</t>
         </is>
       </c>
       <c r="C771" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:57:47 +0700</t>
+          <t>Tue, 04 Aug 2026 21:43:26 +0700</t>
         </is>
       </c>
       <c r="D771" t="inlineStr"/>
       <c r="E771" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) menahan tiga tersangka kasus dugaan korupsi dalam pengadaan digitalisasi stasiun ...</t>
+          <t>Indonesia menambah tiga medali yang terdiri dari satu perak dan dua perunggu pada hari keempat 8th Asian Taekwondo ...</t>
         </is>
       </c>
       <c r="F771" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679803/kpk-tahan-tiga-tersangka-kasus-dugaan-korupsi-dalam-digitalisasi-spbu</t>
+          <t>https://www.antaranews.com/berita/5679989/indonesia-tambah-tiga-medali-pada-hari-keempat-indonesia-open</t>
         </is>
       </c>
       <c r="G771" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/konpres-penahanan-tersangka-kasus-korupsi-digitalisasi-spbu-pertamina-2834421_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/adrian-kaiser-raih-perak-asian-taekwondo-indonesia-open-championships-2834348.jpg</t>
         </is>
       </c>
       <c r="H771" t="inlineStr">
@@ -25644,28 +25644,28 @@
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>KMP Mutiara Sentosa; Keselamatan dan pentingnya memanusiakan penumpang</t>
+          <t>KPK tahan tiga tersangka kasus dugaan korupsi dalam digitalisasi SPBU</t>
         </is>
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:55:59 +0700</t>
+          <t>Tue, 04 Aug 2026 19:57:47 +0700</t>
         </is>
       </c>
       <c r="D772" t="inlineStr"/>
       <c r="E772" t="inlineStr">
         <is>
-          <t>Peristiwa terbakarnya Kapal Motor Penyeberangan (KMP) Mutiara Sentosa 2 rute Surabaya-Makassar, pada Minggu (2/8) ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menahan tiga tersangka kasus dugaan korupsi dalam pengadaan digitalisasi stasiun ...</t>
         </is>
       </c>
       <c r="F772" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679800/kmp-mutiara-sentosa-keselamatan-dan-pentingnya-memanusiakan-penumpang</t>
+          <t>https://www.antaranews.com/berita/5679803/kpk-tahan-tiga-tersangka-kasus-dugaan-korupsi-dalam-digitalisasi-spbu</t>
         </is>
       </c>
       <c r="G772" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/KMPMutiara_copy_1280x853.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/konpres-penahanan-tersangka-kasus-korupsi-digitalisasi-spbu-pertamina-2834421_1.jpg</t>
         </is>
       </c>
       <c r="H772" t="inlineStr">
@@ -25682,28 +25682,28 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>Kejagung respons gugatan praperadilan Febrie Adriansyah</t>
+          <t>KMP Mutiara Sentosa; Keselamatan dan pentingnya memanusiakan penumpang</t>
         </is>
       </c>
       <c r="C773" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:03:18 +0700</t>
+          <t>Tue, 04 Aug 2026 19:55:59 +0700</t>
         </is>
       </c>
       <c r="D773" t="inlineStr"/>
       <c r="E773" t="inlineStr">
         <is>
-          <t>Kejaksaan Agung (Kejagung) merespons soal gugatan praperadilan yang akan diajukan tersangka kasus dugaan tindak pidana ...</t>
+          <t>Peristiwa terbakarnya Kapal Motor Penyeberangan (KMP) Mutiara Sentosa 2 rute Surabaya-Makassar, pada Minggu (2/8) ...</t>
         </is>
       </c>
       <c r="F773" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679675/kejagung-respons-gugatan-praperadilan-febrie-adriansyah</t>
+          <t>https://www.antaranews.com/berita/5679800/kmp-mutiara-sentosa-keselamatan-dan-pentingnya-memanusiakan-penumpang</t>
         </is>
       </c>
       <c r="G773" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087161_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/KMPMutiara_copy_1280x853.jpg</t>
         </is>
       </c>
       <c r="H773" t="inlineStr">
@@ -25715,33 +25715,33 @@
     <row r="774">
       <c r="A774" t="inlineStr">
         <is>
-          <t>ekonomi-bursa, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>OJK bentuk Satgas guna siapkan pengaturan dan pengawasan bursa mineral</t>
+          <t>Kejagung respons gugatan praperadilan Febrie Adriansyah</t>
         </is>
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 18:27:14 +0700</t>
+          <t>Tue, 04 Aug 2026 19:03:18 +0700</t>
         </is>
       </c>
       <c r="D774" t="inlineStr"/>
       <c r="E774" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) telah membentuk Satuan Tugas Persiapan Pengaturan dan Pengawasan Bursa Mineral dan ...</t>
+          <t>Kejaksaan Agung (Kejagung) merespons soal gugatan praperadilan yang akan diajukan tersangka kasus dugaan tindak pidana ...</t>
         </is>
       </c>
       <c r="F774" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679619/ojk-bentuk-satgas-guna-siapkan-pengaturan-dan-pengawasan-bursa-mineral</t>
+          <t>https://www.antaranews.com/berita/5679675/kejagung-respons-gugatan-praperadilan-febrie-adriansyah</t>
         </is>
       </c>
       <c r="G774" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.20.41.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087161_1.jpg</t>
         </is>
       </c>
       <c r="H774" t="inlineStr">
@@ -25753,33 +25753,33 @@
     <row r="775">
       <c r="A775" t="inlineStr">
         <is>
-          <t>photo, top-news</t>
+          <t>ekonomi-bursa, top-news</t>
         </is>
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>Latihan musik Pagelaran Sabang Merauke</t>
+          <t>OJK bentuk Satgas guna siapkan pengaturan dan pengawasan bursa mineral</t>
         </is>
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 18:18:17 +0700</t>
+          <t>Tue, 04 Aug 2026 18:27:14 +0700</t>
         </is>
       </c>
       <c r="D775" t="inlineStr"/>
       <c r="E775" t="inlineStr">
         <is>
-          <t>Penampilan Yura Yunita (kiri) bersama vokalis Padi Reborn Andi Fadly Arifuddin (kanan) pada latihan musik Pagelaran ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) telah membentuk Satuan Tugas Persiapan Pengaturan dan Pengawasan Bursa Mineral dan ...</t>
         </is>
       </c>
       <c r="F775" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5679585/latihan-musik-pagelaran-sabang-merauke</t>
+          <t>https://www.antaranews.com/berita/5679619/ojk-bentuk-satgas-guna-siapkan-pengaturan-dan-pengawasan-bursa-mineral</t>
         </is>
       </c>
       <c r="G775" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/latihan-musik-pagelaran-sabang-merauke-040826-dr-04.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.20.41.jpeg</t>
         </is>
       </c>
       <c r="H775" t="inlineStr">
@@ -25791,33 +25791,33 @@
     <row r="776">
       <c r="A776" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>photo, top-news</t>
         </is>
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>Kemenkes: Anak harus dilindungi dari promosi vape di medsos</t>
+          <t>Latihan musik Pagelaran Sabang Merauke</t>
         </is>
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 18:14:32 +0700</t>
+          <t>Tue, 04 Aug 2026 18:18:17 +0700</t>
         </is>
       </c>
       <c r="D776" t="inlineStr"/>
       <c r="E776" t="inlineStr">
         <is>
-          <t>Kementerian Kesehatan menegaskan bahwa anak harus dilindungi dari paparan dan promosi produk tembakau, baik ...</t>
+          <t>Penampilan Yura Yunita (kiri) bersama vokalis Padi Reborn Andi Fadly Arifuddin (kanan) pada latihan musik Pagelaran ...</t>
         </is>
       </c>
       <c r="F776" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679575/kemenkes-anak-harus-dilindungi-dari-promosi-vape-di-medsos</t>
+          <t>https://www.antaranews.com/foto/5679585/latihan-musik-pagelaran-sabang-merauke</t>
         </is>
       </c>
       <c r="G776" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/10/usulan-pelarangan-rokok-elektronik-di-ruu-narkotika-2768977.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/latihan-musik-pagelaran-sabang-merauke-040826-dr-04.jpg</t>
         </is>
       </c>
       <c r="H776" t="inlineStr">
@@ -25829,33 +25829,33 @@
     <row r="777">
       <c r="A777" t="inlineStr">
         <is>
-          <t>ekonomi-bursa, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>OJK: Arus dana asing berbalik positif "net buy" Rp1,62 triliun di Juli</t>
+          <t>Kemenkes: Anak harus dilindungi dari promosi vape di medsos</t>
         </is>
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 17:36:42 +0700</t>
+          <t>Tue, 04 Aug 2026 18:14:32 +0700</t>
         </is>
       </c>
       <c r="D777" t="inlineStr"/>
       <c r="E777" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mencatat aliran dana investor asing berbalik positif dengan membukukan net buy senilai ...</t>
+          <t>Kementerian Kesehatan menegaskan bahwa anak harus dilindungi dari paparan dan promosi produk tembakau, baik ...</t>
         </is>
       </c>
       <c r="F777" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679520/ojk-arus-dana-asing-berbalik-positif-net-buy-rp162-triliun-di-juli</t>
+          <t>https://www.antaranews.com/berita/5679575/kemenkes-anak-harus-dilindungi-dari-promosi-vape-di-medsos</t>
         </is>
       </c>
       <c r="G777" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/hasan.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/10/usulan-pelarangan-rokok-elektronik-di-ruu-narkotika-2768977.jpg</t>
         </is>
       </c>
       <c r="H777" t="inlineStr">
@@ -25867,33 +25867,33 @@
     <row r="778">
       <c r="A778" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-bursa, top-news</t>
         </is>
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>Jaksa Agung berhentikan sementara status jaksa Febrie Adriansyah</t>
+          <t>OJK: Arus dana asing berbalik positif "net buy" Rp1,62 triliun di Juli</t>
         </is>
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 17:28:52 +0700</t>
+          <t>Tue, 04 Aug 2026 17:36:42 +0700</t>
         </is>
       </c>
       <c r="D778" t="inlineStr"/>
       <c r="E778" t="inlineStr">
         <is>
-          <t>Jaksa Agung RI ST Burhanuddin memberhentikan sementara status jaksa dari mantan Jaksa Agung Muda Bidang Tindak Pidana ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mencatat aliran dana investor asing berbalik positif dengan membukukan net buy senilai ...</t>
         </is>
       </c>
       <c r="F778" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679508/jaksa-agung-berhentikan-sementara-status-jaksa-febrie-adriansyah</t>
+          <t>https://www.antaranews.com/berita/5679520/ojk-arus-dana-asing-berbalik-positif-net-buy-rp162-triliun-di-juli</t>
         </is>
       </c>
       <c r="G778" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087161_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/hasan.jpg</t>
         </is>
       </c>
       <c r="H778" t="inlineStr">
@@ -25910,28 +25910,28 @@
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>Tiga korban TPPO di Libya alami eksploitasi ekonomi</t>
+          <t>Jaksa Agung berhentikan sementara status jaksa Febrie Adriansyah</t>
         </is>
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 16:17:19 +0700</t>
+          <t>Tue, 04 Aug 2026 17:28:52 +0700</t>
         </is>
       </c>
       <c r="D779" t="inlineStr"/>
       <c r="E779" t="inlineStr">
         <is>
-          <t>Ketiga korban Tindak Pidana Perdagangan Orang (TPPO) berinisial NAR (21), SS (45), dan NKR (39) mengalami ...</t>
+          <t>Jaksa Agung RI ST Burhanuddin memberhentikan sementara status jaksa dari mantan Jaksa Agung Muda Bidang Tindak Pidana ...</t>
         </is>
       </c>
       <c r="F779" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679340/tiga-korban-tppo-di-libya-alami-eksploitasi-ekonomi</t>
+          <t>https://www.antaranews.com/berita/5679508/jaksa-agung-berhentikan-sementara-status-jaksa-febrie-adriansyah</t>
         </is>
       </c>
       <c r="G779" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/tiga-korban-tppo-libya-dipulangkan-ke-indonesia-2834140_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000087161_1.jpg</t>
         </is>
       </c>
       <c r="H779" t="inlineStr">
@@ -25948,28 +25948,28 @@
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>PM Thailand: ASEAN kini di persimpangan jalan hadapi tantangan global</t>
+          <t>Tiga korban TPPO di Libya alami eksploitasi ekonomi</t>
         </is>
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 16:11:35 +0700</t>
+          <t>Tue, 04 Aug 2026 16:17:19 +0700</t>
         </is>
       </c>
       <c r="D780" t="inlineStr"/>
       <c r="E780" t="inlineStr">
         <is>
-          <t>Perdana Menteri (PM) Thailand Anutin Charnvirakul mengatakan ASEAN kini berada di persimpangan jalan, dimana pilihan ...</t>
+          <t>Ketiga korban Tindak Pidana Perdagangan Orang (TPPO) berinisial NAR (21), SS (45), dan NKR (39) mengalami ...</t>
         </is>
       </c>
       <c r="F780" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679317/pm-thailand-asean-kini-di-persimpangan-jalan-hadapi-tantangan-global</t>
+          <t>https://www.antaranews.com/berita/5679340/tiga-korban-tppo-di-libya-alami-eksploitasi-ekonomi</t>
         </is>
       </c>
       <c r="G780" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/kunjungan-pm-thailand-ke-sekretariat-asean-2833977_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/tiga-korban-tppo-libya-dipulangkan-ke-indonesia-2834140_1.jpg</t>
         </is>
       </c>
       <c r="H780" t="inlineStr">
@@ -25986,28 +25986,28 @@
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>Penjualan mobil naik, Menkeu yakin daya beli domestik tetap terjaga</t>
+          <t>PM Thailand: ASEAN kini di persimpangan jalan hadapi tantangan global</t>
         </is>
       </c>
       <c r="C781" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 13:45:23 +0700</t>
+          <t>Tue, 04 Aug 2026 16:11:35 +0700</t>
         </is>
       </c>
       <c r="D781" t="inlineStr"/>
       <c r="E781" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan pertumbuhan penjualan mobil menjadi salah satu indikator yang ...</t>
+          <t>Perdana Menteri (PM) Thailand Anutin Charnvirakul mengatakan ASEAN kini berada di persimpangan jalan, dimana pilihan ...</t>
         </is>
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679033/penjualan-mobil-naik-menkeu-yakin-daya-beli-domestik-tetap-terjaga</t>
+          <t>https://www.antaranews.com/berita/5679317/pm-thailand-asean-kini-di-persimpangan-jalan-hadapi-tantangan-global</t>
         </is>
       </c>
       <c r="G781" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-13.13.50.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/kunjungan-pm-thailand-ke-sekretariat-asean-2833977_1.jpg</t>
         </is>
       </c>
       <c r="H781" t="inlineStr">
@@ -26024,28 +26024,28 @@
       </c>
       <c r="B782" t="inlineStr">
         <is>
-          <t>Ada 2 bibit siklon tropis, BMKG: Waspada ombak setinggi 4 meter di RI</t>
+          <t>Penjualan mobil naik, Menkeu yakin daya beli domestik tetap terjaga</t>
         </is>
       </c>
       <c r="C782" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 12:09:44 +0700</t>
+          <t>Tue, 04 Aug 2026 13:45:23 +0700</t>
         </is>
       </c>
       <c r="D782" t="inlineStr"/>
       <c r="E782" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi kemunculan dua bibit siklon tropis sekaligus di wilayah ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan pertumbuhan penjualan mobil menjadi salah satu indikator yang ...</t>
         </is>
       </c>
       <c r="F782" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678879/ada-2-bibit-siklon-tropis-bmkg-waspada-ombak-setinggi-4-meter-di-ri</t>
+          <t>https://www.antaranews.com/berita/5679033/penjualan-mobil-naik-menkeu-yakin-daya-beli-domestik-tetap-terjaga</t>
         </is>
       </c>
       <c r="G782" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_20250609_135328.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-13.13.50.jpg</t>
         </is>
       </c>
       <c r="H782" t="inlineStr">
@@ -26062,28 +26062,28 @@
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>Korban tewas gempa Venezuela terus bertambah jadi 6.100 orang</t>
+          <t>Ada 2 bibit siklon tropis, BMKG: Waspada ombak setinggi 4 meter di RI</t>
         </is>
       </c>
       <c r="C783" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 12:00:56 +0700</t>
+          <t>Tue, 04 Aug 2026 12:09:44 +0700</t>
         </is>
       </c>
       <c r="D783" t="inlineStr"/>
       <c r="E783" t="inlineStr">
         <is>
-          <t>Jumlah korban tewas akibat gempa kembar dahsyat yang mengguncang Venezuela pada 24 Juni 2026, terus bertambah ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi kemunculan dua bibit siklon tropis sekaligus di wilayah ...</t>
         </is>
       </c>
       <c r="F783" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678865/korban-tewas-gempa-venezuela-terus-bertambah-jadi-6100-orang</t>
+          <t>https://www.antaranews.com/berita/5678879/ada-2-bibit-siklon-tropis-bmkg-waspada-ombak-setinggi-4-meter-di-ri</t>
         </is>
       </c>
       <c r="G783" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/thumbs_b_c_d4a34a165f13a0667255577d3cfac46f.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_20250609_135328.jpg</t>
         </is>
       </c>
       <c r="H783" t="inlineStr">
@@ -26100,28 +26100,28 @@
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>BPKH salurkan Rp2,06 triliun nilai manfaat ke 5,7 juta calon haji</t>
+          <t>Korban tewas gempa Venezuela terus bertambah jadi 6.100 orang</t>
         </is>
       </c>
       <c r="C784" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 11:47:58 +0700</t>
+          <t>Tue, 04 Aug 2026 12:00:56 +0700</t>
         </is>
       </c>
       <c r="D784" t="inlineStr"/>
       <c r="E784" t="inlineStr">
         <is>
-          <t>Badan Pengelola Keuangan Haji (BPKH) menyalurkan Nilai Manfaat Tahap I Tahun 2026 lebih dari Rp2,06 triliun kepada ...</t>
+          <t>Jumlah korban tewas akibat gempa kembar dahsyat yang mengguncang Venezuela pada 24 Juni 2026, terus bertambah ...</t>
         </is>
       </c>
       <c r="F784" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678849/bpkh-salurkan-rp206-triliun-nilai-manfaat-ke-57-juta-calon-haji</t>
+          <t>https://www.antaranews.com/berita/5678865/korban-tewas-gempa-venezuela-terus-bertambah-jadi-6100-orang</t>
         </is>
       </c>
       <c r="G784" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000176506_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/thumbs_b_c_d4a34a165f13a0667255577d3cfac46f.jpg</t>
         </is>
       </c>
       <c r="H784" t="inlineStr">
@@ -26138,28 +26138,28 @@
       </c>
       <c r="B785" t="inlineStr">
         <is>
-          <t>Aldila jadi petenis Indonesia yang pertama juarai DC Open</t>
+          <t>BPKH salurkan Rp2,06 triliun nilai manfaat ke 5,7 juta calon haji</t>
         </is>
       </c>
       <c r="C785" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 11:39:37 +0700</t>
+          <t>Tue, 04 Aug 2026 11:47:58 +0700</t>
         </is>
       </c>
       <c r="D785" t="inlineStr"/>
       <c r="E785" t="inlineStr">
         <is>
-          <t>Petenis Indonesia Aldila Sutjiadi mencatatkan sejarah setelah menjuarai nomor ganda putri turnamen Mubadala DC Open ...</t>
+          <t>Badan Pengelola Keuangan Haji (BPKH) menyalurkan Nilai Manfaat Tahap I Tahun 2026 lebih dari Rp2,06 triliun kepada ...</t>
         </is>
       </c>
       <c r="F785" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678836/aldila-jadi-petenis-indonesia-yang-pertama-juarai-dc-open</t>
+          <t>https://www.antaranews.com/berita/5678849/bpkh-salurkan-rp206-triliun-nilai-manfaat-ke-57-juta-calon-haji</t>
         </is>
       </c>
       <c r="G785" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_4155-copy.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000176506_1.jpg</t>
         </is>
       </c>
       <c r="H785" t="inlineStr">
@@ -26176,28 +26176,28 @@
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>Indonesia raih 15 medali dari Kejuaraan MMAAsia</t>
+          <t>Aldila jadi petenis Indonesia yang pertama juarai DC Open</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 09:16:36 +0700</t>
+          <t>Tue, 04 Aug 2026 11:39:37 +0700</t>
         </is>
       </c>
       <c r="D786" t="inlineStr"/>
       <c r="E786" t="inlineStr">
         <is>
-          <t>Tim mixed martial arts (MMA) amatir Indonesia meraih 15 medali dan menempati peringkat keempat pada GAMMA Asian ...</t>
+          <t>Petenis Indonesia Aldila Sutjiadi mencatatkan sejarah setelah menjuarai nomor ganda putri turnamen Mubadala DC Open ...</t>
         </is>
       </c>
       <c r="F786" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678689/indonesia-raih-15-medali-dari-kejuaraan-mmaasia</t>
+          <t>https://www.antaranews.com/berita/5678836/aldila-jadi-petenis-indonesia-yang-pertama-juarai-dc-open</t>
         </is>
       </c>
       <c r="G786" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Delvi-Novia_Medal.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_4155-copy.jpg</t>
         </is>
       </c>
       <c r="H786" t="inlineStr">
@@ -26214,28 +26214,28 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>Kontingen Indonesia di Asian Games 2026</t>
+          <t>Indonesia raih 15 medali dari Kejuaraan MMAAsia</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 06:00:00 +0700</t>
+          <t>Tue, 04 Aug 2026 09:16:36 +0700</t>
         </is>
       </c>
       <c r="D787" t="inlineStr"/>
       <c r="E787" t="inlineStr">
         <is>
-          <t>Indonesia mengirimkan 432 atlet terbaik untuk berlaga di Asian Games 2026 pada 19 September-4 Oktober di Aichi dan ...</t>
+          <t>Tim mixed martial arts (MMA) amatir Indonesia meraih 15 medali dan menempati peringkat keempat pada GAMMA Asian ...</t>
         </is>
       </c>
       <c r="F787" t="inlineStr">
         <is>
-          <t>https://asiangames.antaranews.com/infografik/5677857/kontingen-indonesia-di-asian-games-2026</t>
+          <t>https://www.antaranews.com/berita/5678689/indonesia-raih-15-medali-dari-kejuaraan-mmaasia</t>
         </is>
       </c>
       <c r="G787" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Kontingen-Indonesia-di-Asian-Games-2026.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/Delvi-Novia_Medal.jpg</t>
         </is>
       </c>
       <c r="H787" t="inlineStr">
@@ -26252,28 +26252,28 @@
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>Rizky Ridho abaikan kritik negatif untuk jaga fokus kontra Singapura</t>
+          <t>Kontingen Indonesia di Asian Games 2026</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 04:45:38 +0700</t>
+          <t>Tue, 04 Aug 2026 06:00:00 +0700</t>
         </is>
       </c>
       <c r="D788" t="inlineStr"/>
       <c r="E788" t="inlineStr">
         <is>
-          <t>Kapten tim nasional sepak bola Indonesia Rizky Ridho memilih mengabaikan kritik negatif terkait penampilannya saat ...</t>
+          <t>Indonesia mengirimkan 432 atlet terbaik untuk berlaga di Asian Games 2026 pada 19 September-4 Oktober di Aichi dan ...</t>
         </is>
       </c>
       <c r="F788" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678603/rizky-ridho-abaikan-kritik-negatif-untuk-jaga-fokus-kontra-singapura</t>
+          <t>https://asiangames.antaranews.com/infografik/5677857/kontingen-indonesia-di-asian-games-2026</t>
         </is>
       </c>
       <c r="G788" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833529.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Kontingen-Indonesia-di-Asian-Games-2026.jpg</t>
         </is>
       </c>
       <c r="H788" t="inlineStr">
@@ -26285,33 +26285,33 @@
     <row r="789">
       <c r="A789" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>Tiket GIIAS 2026: Daftar Harga dan cara belinya</t>
+          <t>Rizky Ridho abaikan kritik negatif untuk jaga fokus kontra Singapura</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 16:29:46 +0700</t>
+          <t>Tue, 04 Aug 2026 04:45:38 +0700</t>
         </is>
       </c>
       <c r="D789" t="inlineStr"/>
       <c r="E789" t="inlineStr">
         <is>
-          <t>Pameran GAIKINDO Indonesia International Auto Show (GIIAS) 2026 resmi digelar sejak 30 Juli hingga 9 Agustus 2026. ...</t>
+          <t>Kapten tim nasional sepak bola Indonesia Rizky Ridho memilih mengabaikan kritik negatif terkait penampilannya saat ...</t>
         </is>
       </c>
       <c r="F789" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5679373/tiket-giias-2026-daftar-harga-dan-cara-belinya</t>
+          <t>https://www.antaranews.com/berita/5678603/rizky-ridho-abaikan-kritik-negatif-untuk-jaga-fokus-kontra-singapura</t>
         </is>
       </c>
       <c r="G789" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/WhatsApp-Image-2026-07-30-at-21.31.47.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833529.jpg</t>
         </is>
       </c>
       <c r="H789" t="inlineStr">
@@ -26323,33 +26323,33 @@
     <row r="790">
       <c r="A790" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Penyidik OJK selesaikan 187 perkara sektor jasa keuangan hingga Juli</t>
+          <t>Tiket GIIAS 2026: Daftar Harga dan cara belinya</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 21:58:58 +0700</t>
+          <t>Tue, 04 Aug 2026 16:29:46 +0700</t>
         </is>
       </c>
       <c r="D790" t="inlineStr"/>
       <c r="E790" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) menyatakan bahwa penyidik OJK telah menyelesaikan total 187 perkara di sektor jasa ...</t>
+          <t>Pameran GAIKINDO Indonesia International Auto Show (GIIAS) 2026 resmi digelar sejak 30 Juli hingga 9 Agustus 2026. ...</t>
         </is>
       </c>
       <c r="F790" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5680011/penyidik-ojk-selesaikan-187-perkara-sektor-jasa-keuangan-hingga-juli</t>
+          <t>https://otomotif.antaranews.com/berita/5679373/tiket-giias-2026-daftar-harga-dan-cara-belinya</t>
         </is>
       </c>
       <c r="G790" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-21.16.28.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/30/WhatsApp-Image-2026-07-30-at-21.31.47.jpeg</t>
         </is>
       </c>
       <c r="H790" t="inlineStr">
@@ -26366,28 +26366,28 @@
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>OJK: IASC memulihkan dana korban penipuan Rp204,3 miliar hingga Juli</t>
+          <t>Penyidik OJK selesaikan 187 perkara sektor jasa keuangan hingga Juli</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 21:29:11 +0700</t>
+          <t>Tue, 04 Aug 2026 21:58:58 +0700</t>
         </is>
       </c>
       <c r="D791" t="inlineStr"/>
       <c r="E791" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) menyampaikan bahwa Indonesia Anti-Scam Centre (IASC) hingga akhir Juli 2026 berhasil ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) menyatakan bahwa penyidik OJK telah menyelesaikan total 187 perkara di sektor jasa ...</t>
         </is>
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679972/ojk-iasc-memulihkan-dana-korban-penipuan-rp2043-miliar-hingga-juli</t>
+          <t>https://www.antaranews.com/berita/5680011/penyidik-ojk-selesaikan-187-perkara-sektor-jasa-keuangan-hingga-juli</t>
         </is>
       </c>
       <c r="G791" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-21.10.24.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-21.16.28.jpeg</t>
         </is>
       </c>
       <c r="H791" t="inlineStr">
@@ -26404,28 +26404,28 @@
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>OJK: Premi industri asuransi capai Rp170,98 triliun di semester I-2026</t>
+          <t>OJK: IASC memulihkan dana korban penipuan Rp204,3 miliar hingga Juli</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 20:41:07 +0700</t>
+          <t>Tue, 04 Aug 2026 21:29:11 +0700</t>
         </is>
       </c>
       <c r="D792" t="inlineStr"/>
       <c r="E792" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan akumulasi pendapatan premi industri asuransi komersil mencapai Rp170,98 triliun ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) menyampaikan bahwa Indonesia Anti-Scam Centre (IASC) hingga akhir Juli 2026 berhasil ...</t>
         </is>
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679872/ojk-premi-industri-asuransi-capai-rp17098-triliun-di-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5679972/ojk-iasc-memulihkan-dana-korban-penipuan-rp2043-miliar-hingga-juli</t>
         </is>
       </c>
       <c r="G792" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/ogi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-21.10.24.jpeg</t>
         </is>
       </c>
       <c r="H792" t="inlineStr">
@@ -26442,28 +26442,28 @@
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>OJK: Target bisnis BPR-BPRS hasil revisi tetap kontributif ke ekonomi</t>
+          <t>OJK: Premi industri asuransi capai Rp170,98 triliun di semester I-2026</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 20:33:27 +0700</t>
+          <t>Tue, 04 Aug 2026 20:41:07 +0700</t>
         </is>
       </c>
       <c r="D793" t="inlineStr"/>
       <c r="E793" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) memandang bahwa target bisnis bank perekonomian rakyat (BPR) dan BPR Syariah (BPRS) hasil ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan akumulasi pendapatan premi industri asuransi komersil mencapai Rp170,98 triliun ...</t>
         </is>
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679857/ojk-target-bisnis-bpr-bprs-hasil-revisi-tetap-kontributif-ke-ekonomi</t>
+          <t>https://www.antaranews.com/berita/5679872/ojk-premi-industri-asuransi-capai-rp17098-triliun-di-semester-i-2026</t>
         </is>
       </c>
       <c r="G793" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.54.16.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/ogi.jpg</t>
         </is>
       </c>
       <c r="H793" t="inlineStr">
@@ -26480,28 +26480,28 @@
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>OJK: IASC terima 1.379 laporan terkait penipuan keuangan berbasis AI</t>
+          <t>OJK: Target bisnis BPR-BPRS hasil revisi tetap kontributif ke ekonomi</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 20:12:26 +0700</t>
+          <t>Tue, 04 Aug 2026 20:33:27 +0700</t>
         </is>
       </c>
       <c r="D794" t="inlineStr"/>
       <c r="E794" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan terdapat 1.379 laporan penipuan keuangan yang terindikasi memanfaatkan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) memandang bahwa target bisnis bank perekonomian rakyat (BPR) dan BPR Syariah (BPRS) hasil ...</t>
         </is>
       </c>
       <c r="F794" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679819/ojk-iasc-terima-1379-laporan-terkait-penipuan-keuangan-berbasis-ai</t>
+          <t>https://www.antaranews.com/berita/5679857/ojk-target-bisnis-bpr-bprs-hasil-revisi-tetap-kontributif-ke-ekonomi</t>
         </is>
       </c>
       <c r="G794" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-20.01.41.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.54.16.jpeg</t>
         </is>
       </c>
       <c r="H794" t="inlineStr">
@@ -26518,28 +26518,28 @@
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>Kementerian PKP: Opini WTP dari BPK dorong anggaran lebih pro rakyat</t>
+          <t>OJK: IASC terima 1.379 laporan terkait penipuan keuangan berbasis AI</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 20:04:22 +0700</t>
+          <t>Tue, 04 Aug 2026 20:12:26 +0700</t>
         </is>
       </c>
       <c r="D795" t="inlineStr"/>
       <c r="E795" t="inlineStr">
         <is>
-          <t>Kementerian Perumahan dan Kawasan Permukiman (PKP) mendapatkan opini Wajar Tanpa Pengecualian (WTP) dari Badan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan terdapat 1.379 laporan penipuan keuangan yang terindikasi memanfaatkan ...</t>
         </is>
       </c>
       <c r="F795" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679812/kementerian-pkp-opini-wtp-dari-bpk-dorong-anggaran-lebih-pro-rakyat</t>
+          <t>https://www.antaranews.com/berita/5679819/ojk-iasc-terima-1379-laporan-terkait-penipuan-keuangan-berbasis-ai</t>
         </is>
       </c>
       <c r="G795" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000590797.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-20.01.41.jpeg</t>
         </is>
       </c>
       <c r="H795" t="inlineStr">
@@ -26556,28 +26556,28 @@
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>OJK catat transaksi kripto capai Rp28,58 triliun pada Juni 2026</t>
+          <t>Kementerian PKP: Opini WTP dari BPK dorong anggaran lebih pro rakyat</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:44:43 +0700</t>
+          <t>Tue, 04 Aug 2026 20:04:22 +0700</t>
         </is>
       </c>
       <c r="D796" t="inlineStr"/>
       <c r="E796" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mencatat nilai transaksi aset kripto di Indonesia mencapai Rp28,58 triliun pada Juni 2026 ...</t>
+          <t>Kementerian Perumahan dan Kawasan Permukiman (PKP) mendapatkan opini Wajar Tanpa Pengecualian (WTP) dari Badan ...</t>
         </is>
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679757/ojk-catat-transaksi-kripto-capai-rp2858-triliun-pada-juni-2026</t>
+          <t>https://www.antaranews.com/berita/5679812/kementerian-pkp-opini-wtp-dari-bpk-dorong-anggaran-lebih-pro-rakyat</t>
         </is>
       </c>
       <c r="G796" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/ojk-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1000590797.jpg</t>
         </is>
       </c>
       <c r="H796" t="inlineStr">
@@ -26594,28 +26594,28 @@
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>Purbaya pastikan penempatan dana pemerintah di Himbara tetap berjalan</t>
+          <t>OJK catat transaksi kripto capai Rp28,58 triliun pada Juni 2026</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:38:01 +0700</t>
+          <t>Tue, 04 Aug 2026 19:44:43 +0700</t>
         </is>
       </c>
       <c r="D797" t="inlineStr"/>
       <c r="E797" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa memastikan penempatan dana pemerintah pada HImpunan Bank Milik Negara (Himbara) ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mencatat nilai transaksi aset kripto di Indonesia mencapai Rp28,58 triliun pada Juni 2026 ...</t>
         </is>
       </c>
       <c r="F797" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679741/purbaya-pastikan-penempatan-dana-pemerintah-di-himbara-tetap-berjalan</t>
+          <t>https://www.antaranews.com/berita/5679757/ojk-catat-transaksi-kripto-capai-rp2858-triliun-pada-juni-2026</t>
         </is>
       </c>
       <c r="G797" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-13.13.50.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/ojk-1.jpg</t>
         </is>
       </c>
       <c r="H797" t="inlineStr">
@@ -26632,28 +26632,28 @@
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>OJK: Baki debet "paylater" tumbuh 33,54 persen, didorong KBMI 1 dan 3</t>
+          <t>Purbaya pastikan penempatan dana pemerintah di Himbara tetap berjalan</t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 19:33:17 +0700</t>
+          <t>Tue, 04 Aug 2026 19:38:01 +0700</t>
         </is>
       </c>
       <c r="D798" t="inlineStr"/>
       <c r="E798" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan baki debet buy now pay later (BNPL) perbankan tumbuh 33,54 persen secara ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa memastikan penempatan dana pemerintah pada HImpunan Bank Milik Negara (Himbara) ...</t>
         </is>
       </c>
       <c r="F798" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679721/ojk-baki-debet-paylater-tumbuh-3354-persen-didorong-kbmi-1-dan-3</t>
+          <t>https://www.antaranews.com/berita/5679741/purbaya-pastikan-penempatan-dana-pemerintah-di-himbara-tetap-berjalan</t>
         </is>
       </c>
       <c r="G798" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.54.16-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-13.13.50.jpg</t>
         </is>
       </c>
       <c r="H798" t="inlineStr">
@@ -26670,28 +26670,28 @@
       </c>
       <c r="B799" t="inlineStr">
         <is>
-          <t>Rupiah melemah dipicu defisit neraca perdagangan Indonesia</t>
+          <t>OJK: Baki debet "paylater" tumbuh 33,54 persen, didorong KBMI 1 dan 3</t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 17:15:39 +0700</t>
+          <t>Tue, 04 Aug 2026 19:33:17 +0700</t>
         </is>
       </c>
       <c r="D799" t="inlineStr"/>
       <c r="E799" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Selasa, bergerak melemah 30 poin atau 0,17 persen ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) mengungkapkan baki debet buy now pay later (BNPL) perbankan tumbuh 33,54 persen secara ...</t>
         </is>
       </c>
       <c r="F799" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679493/rupiah-melemah-dipicu-defisit-neraca-perdagangan-indonesia</t>
+          <t>https://www.antaranews.com/berita/5679721/ojk-baki-debet-paylater-tumbuh-3354-persen-didorong-kbmi-1-dan-3</t>
         </is>
       </c>
       <c r="G799" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/1000680361.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-18.54.16-1.jpeg</t>
         </is>
       </c>
       <c r="H799" t="inlineStr">
@@ -26708,28 +26708,28 @@
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>Krom Bank perkuat kerja sama pembiayaan dengan Pandai Gadai</t>
+          <t>Rupiah melemah dipicu defisit neraca perdagangan Indonesia</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 16:37:21 +0700</t>
+          <t>Tue, 04 Aug 2026 17:15:39 +0700</t>
         </is>
       </c>
       <c r="D800" t="inlineStr"/>
       <c r="E800" t="inlineStr">
         <is>
-          <t>PT Krom Bank Indonesia Tbk (Kode emiten: BBSI), memperkuat kemitraan pembiayaannya dengan memberikan fasilitas kredit ...</t>
+          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Selasa, bergerak melemah 30 poin atau 0,17 persen ...</t>
         </is>
       </c>
       <c r="F800" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679393/krom-bank-perkuat-kerja-sama-pembiayaan-dengan-pandai-gadai</t>
+          <t>https://www.antaranews.com/berita/5679493/rupiah-melemah-dipicu-defisit-neraca-perdagangan-indonesia</t>
         </is>
       </c>
       <c r="G800" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-2.14.24-PM.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/1000680361.jpg</t>
         </is>
       </c>
       <c r="H800" t="inlineStr">
@@ -26746,28 +26746,28 @@
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>OJK luncurkan 12.969 rekening "Simpel" perluas akses keuangan pelajar</t>
+          <t>Krom Bank perkuat kerja sama pembiayaan dengan Pandai Gadai</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 16:07:32 +0700</t>
+          <t>Tue, 04 Aug 2026 16:37:21 +0700</t>
         </is>
       </c>
       <c r="D801" t="inlineStr"/>
       <c r="E801" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) Sulawesi Tenggara (Sultra) bersama pemerintah kabupaten dan PT BPR Bahteramas Konawe ...</t>
+          <t>PT Krom Bank Indonesia Tbk (Kode emiten: BBSI), memperkuat kemitraan pembiayaannya dengan memberikan fasilitas kredit ...</t>
         </is>
       </c>
       <c r="F801" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679311/ojk-luncurkan-12969-rekening-simpel-perluas-akses-keuangan-pelajar</t>
+          <t>https://www.antaranews.com/berita/5679393/krom-bank-perkuat-kerja-sama-pembiayaan-dengan-pandai-gadai</t>
         </is>
       </c>
       <c r="G801" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_1266.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-2.14.24-PM.jpeg</t>
         </is>
       </c>
       <c r="H801" t="inlineStr">
@@ -26784,28 +26784,28 @@
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
+          <t>OJK luncurkan 12.969 rekening "Simpel" perluas akses keuangan pelajar</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 15:41:45 +0700</t>
+          <t>Tue, 04 Aug 2026 16:07:32 +0700</t>
         </is>
       </c>
       <c r="D802" t="inlineStr"/>
       <c r="E802" t="inlineStr">
         <is>
-          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) Sulawesi Tenggara (Sultra) bersama pemerintah kabupaten dan PT BPR Bahteramas Konawe ...</t>
         </is>
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
+          <t>https://www.antaranews.com/berita/5679311/ojk-luncurkan-12969-rekening-simpel-perluas-akses-keuangan-pelajar</t>
         </is>
       </c>
       <c r="G802" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_1266.jpeg</t>
         </is>
       </c>
       <c r="H802" t="inlineStr">
@@ -26822,28 +26822,28 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Bappenas: Presiden minta soal iklim tIdak ganggu stabilitas nasional</t>
+          <t>Indonesia-Thailand gelar forum bisnis tingkatkan kerja sama ekonomi</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 14:47:39 +0700</t>
+          <t>Tue, 04 Aug 2026 15:41:45 +0700</t>
         </is>
       </c>
       <c r="D803" t="inlineStr"/>
       <c r="E803" t="inlineStr">
         <is>
-          <t>Menteri Perencanaan Pembangunan Nasional (PPN)/Kepala Badan Perencanaan Pembangunan Nasional (Bappenas) Rachmat Pambudy ...</t>
+          <t>ANTARA - Kamar Dagang dan Industri (Kadin) Indonesia menggelar Indonesia-Thailand Bisnis Forum di Jakarta pada Selasa ...</t>
         </is>
       </c>
       <c r="F803" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679137/bappenas-presiden-minta-soal-iklim-tidak-ganggu-stabilitas-nasional</t>
+          <t>https://www.antaranews.com/video/5679221/indonesia-thailand-gelar-forum-bisnis-tingkatkan-kerja-sama-ekonomi</t>
         </is>
       </c>
       <c r="G803" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-14.11.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-THAILAND-GELAR-FORUM-BISNIS-TINGKATKAN-KERJA-SAMA-EKONOMI.jpg</t>
         </is>
       </c>
       <c r="H803" t="inlineStr">
@@ -26860,28 +26860,28 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>Ekonom: Pasokan pangan membaik jaga inflasi tetap terkendali</t>
+          <t>Bappenas: Presiden minta soal iklim tIdak ganggu stabilitas nasional</t>
         </is>
       </c>
       <c r="C804" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 14:23:45 +0700</t>
+          <t>Tue, 04 Aug 2026 14:47:39 +0700</t>
         </is>
       </c>
       <c r="D804" t="inlineStr"/>
       <c r="E804" t="inlineStr">
         <is>
-          <t>Ekonom PT Bank Danamon Indonesia Tbk menilai inflasi pada Juli 2026 tetap terkendali seiring membaiknya pasokan pangan ...</t>
+          <t>Menteri Perencanaan Pembangunan Nasional (PPN)/Kepala Badan Perencanaan Pembangunan Nasional (Bappenas) Rachmat Pambudy ...</t>
         </is>
       </c>
       <c r="F804" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5679091/ekonom-pasokan-pangan-membaik-jaga-inflasi-tetap-terkendali</t>
+          <t>https://www.antaranews.com/berita/5679137/bappenas-presiden-minta-soal-iklim-tidak-ganggu-stabilitas-nasional</t>
         </is>
       </c>
       <c r="G804" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/inflasi-juli-2026-jawa-barat-2833080.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-14.11.29.jpeg</t>
         </is>
       </c>
       <c r="H804" t="inlineStr">
@@ -26898,28 +26898,28 @@
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>LPEM FEB UI perkirakan ekonomi RI tumbuh 4,8 persen di kuartal II 2026</t>
+          <t>Ekonom: Pasokan pangan membaik jaga inflasi tetap terkendali</t>
         </is>
       </c>
       <c r="C805" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 12:57:01 +0700</t>
+          <t>Tue, 04 Aug 2026 14:23:45 +0700</t>
         </is>
       </c>
       <c r="D805" t="inlineStr"/>
       <c r="E805" t="inlineStr">
         <is>
-          <t>Lembaga Penyelidikan Ekonomi dan Masyarakat Fakultas Ekonomi dan Bisnis Universitas Indonesia (LPEM FEB UI) ...</t>
+          <t>Ekonom PT Bank Danamon Indonesia Tbk menilai inflasi pada Juli 2026 tetap terkendali seiring membaiknya pasokan pangan ...</t>
         </is>
       </c>
       <c r="F805" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678945/lpem-feb-ui-perkirakan-ekonomi-ri-tumbuh-48-persen-di-kuartal-ii-2026</t>
+          <t>https://www.antaranews.com/berita/5679091/ekonom-pasokan-pangan-membaik-jaga-inflasi-tetap-terkendali</t>
         </is>
       </c>
       <c r="G805" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2022/05/17/Screenshot_20220517-151559_YouTube.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/inflasi-juli-2026-jawa-barat-2833080.jpg</t>
         </is>
       </c>
       <c r="H805" t="inlineStr">
@@ -26936,28 +26936,28 @@
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>BI siapkan Rp20 miliar ekspedisi rupiah berdaulat 2026 di 3T Papua</t>
+          <t>LPEM FEB UI perkirakan ekonomi RI tumbuh 4,8 persen di kuartal II 2026</t>
         </is>
       </c>
       <c r="C806" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 12:24:47 +0700</t>
+          <t>Tue, 04 Aug 2026 12:57:01 +0700</t>
         </is>
       </c>
       <c r="D806" t="inlineStr"/>
       <c r="E806" t="inlineStr">
         <is>
-          <t>Kantor Perwakilan Bank Indonesia (BI) Provinsi Papua menyiapkan uang layak edar senilai Rp20 miliar dalam pelaksanaan ...</t>
+          <t>Lembaga Penyelidikan Ekonomi dan Masyarakat Fakultas Ekonomi dan Bisnis Universitas Indonesia (LPEM FEB UI) ...</t>
         </is>
       </c>
       <c r="F806" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678896/bi-siapkan-rp20-miliar-ekspedisi-rupiah-berdaulat-2026-di-3t-papua</t>
+          <t>https://www.antaranews.com/berita/5678945/lpem-feb-ui-perkirakan-ekonomi-ri-tumbuh-48-persen-di-kuartal-ii-2026</t>
         </is>
       </c>
       <c r="G806" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1002062154.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/05/17/Screenshot_20220517-151559_YouTube.jpg</t>
         </is>
       </c>
       <c r="H806" t="inlineStr">
@@ -26974,28 +26974,28 @@
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>Panda Bond dan sinyal kepercayaan investasi global</t>
+          <t>BI siapkan Rp20 miliar ekspedisi rupiah berdaulat 2026 di 3T Papua</t>
         </is>
       </c>
       <c r="C807" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 11:26:35 +0700</t>
+          <t>Tue, 04 Aug 2026 12:24:47 +0700</t>
         </is>
       </c>
       <c r="D807" t="inlineStr"/>
       <c r="E807" t="inlineStr">
         <is>
-          <t>Di tengah ketidakpastian ekonomi global yang semakin kompleks, pemerintah Indonesia perlu memastikan bahwa ...</t>
+          <t>Kantor Perwakilan Bank Indonesia (BI) Provinsi Papua menyiapkan uang layak edar senilai Rp20 miliar dalam pelaksanaan ...</t>
         </is>
       </c>
       <c r="F807" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678827/panda-bond-dan-sinyal-kepercayaan-investasi-global</t>
+          <t>https://www.antaranews.com/berita/5678896/bi-siapkan-rp20-miliar-ekspedisi-rupiah-berdaulat-2026-di-3t-papua</t>
         </is>
       </c>
       <c r="G807" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/15/permintaan-pembelian-obligasi-global-capai-46-miliar-dolar-as-2806089.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/1002062154.jpg</t>
         </is>
       </c>
       <c r="H807" t="inlineStr">
@@ -27012,28 +27012,28 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Rupiah Selasa melemah dipicu kenaikan harga minyak global</t>
+          <t>Panda Bond dan sinyal kepercayaan investasi global</t>
         </is>
       </c>
       <c r="C808" t="inlineStr">
         <is>
-          <t>Tue, 04 Aug 2026 11:15:57 +0700</t>
+          <t>Tue, 04 Aug 2026 11:26:35 +0700</t>
         </is>
       </c>
       <c r="D808" t="inlineStr"/>
       <c r="E808" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah pada Selasa pagi bergerak melemah 32 poin atau 0,18 persen menjadi Rp18.029 per dolar AS ...</t>
+          <t>Di tengah ketidakpastian ekonomi global yang semakin kompleks, pemerintah Indonesia perlu memastikan bahwa ...</t>
         </is>
       </c>
       <c r="F808" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678808/rupiah-selasa-melemah-dipicu-kenaikan-harga-minyak-global</t>
+          <t>https://www.antaranews.com/berita/5678827/panda-bond-dan-sinyal-kepercayaan-investasi-global</t>
         </is>
       </c>
       <c r="G808" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/13/nilai-tukar-rupiah-melemah-44-poin-2821215.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/15/permintaan-pembelian-obligasi-global-capai-46-miliar-dolar-as-2806089.jpg</t>
         </is>
       </c>
       <c r="H808" t="inlineStr">

</xml_diff>